<commit_message>
style(brand): enforce Etazhi corporate colors (Red, Gray, White) across MASTER_LOG and AGENTS.md guidelines
</commit_message>
<xml_diff>
--- a/MASTER_LOG.xlsx
+++ b/MASTER_LOG.xlsx
@@ -33,7 +33,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001E3A8A"/>
+      <color rgb="00C8102E"/>
       <sz val="15"/>
     </font>
     <font>
@@ -67,14 +67,15 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="002563EB"/>
+      <b val="1"/>
+      <color rgb="00C8102E"/>
       <sz val="10"/>
       <u val="single"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00991B1B"/>
+      <color rgb="00C8102E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -84,7 +85,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -93,8 +94,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
+        <fgColor rgb="00C8102E"/>
+        <bgColor rgb="00C8102E"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,12 +130,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
@@ -150,16 +145,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00FFFFFF"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00FFFFFF"/>
       </right>
       <top style="medium">
-        <color rgb="001E3A8A"/>
+        <color rgb="00990000"/>
       </top>
       <bottom style="medium">
-        <color rgb="001E3A8A"/>
+        <color rgb="00990000"/>
       </bottom>
     </border>
     <border>
@@ -235,12 +230,12 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -637,7 +632,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Нажмите на кнопку [+] над столбцами I-M, чтобы раскрыть подробные реквизиты и проверки (Паспорт, ИНН, Адрес, Арбитраж, Суды, РСФН)</t>
+          <t>Нажмите на кнопку [+] над столбцами I-M, чтобы раскрыть подробные реквизиты (Паспорт, ИНН, Адрес, Арбитраж, Суды, РСФН)</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2457,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Компактная таблица основных параметров. Детальные проверки по каждому стажеру вынесены на отдельную вкладку «Карточка досье».</t>
+          <t>Компактная таблица основных параметров. Детальные проверки по каждому стажеру вынесены на вкладку «Карточки досье».</t>
         </is>
       </c>
     </row>

</xml_diff>